<commit_message>
Update DevSim application and templates
</commit_message>
<xml_diff>
--- a/DevSim/Active/Network Settings.xlsx
+++ b/DevSim/Active/Network Settings.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/glennshields/Desktop/NewTemplates/Default_DevSim_Template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/glennshields/Desktop/DevSim/Active/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BDE6587-22D2-6949-A617-F368A25F734D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23BC4531-371E-D441-9AC2-4345BBF2C459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="300" yWindow="760" windowWidth="27520" windowHeight="18960" xr2:uid="{D5439726-C23F-F743-B6C6-59C619D7D47A}"/>
+    <workbookView xWindow="30240" yWindow="2220" windowWidth="27520" windowHeight="18960" activeTab="1" xr2:uid="{D5439726-C23F-F743-B6C6-59C619D7D47A}"/>
   </bookViews>
   <sheets>
     <sheet name="Gene Information" sheetId="5" r:id="rId1"/>

</xml_diff>